<commit_message>
modified the mmr_results to have all tabs required for multiple analysis
</commit_message>
<xml_diff>
--- a/src/Data/mmr_results.xlsx
+++ b/src/Data/mmr_results.xlsx
@@ -7,7 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="general_immunity" sheetId="1" r:id="rId1"/>
+    <sheet name="population_immunity" sheetId="2" r:id="rId2"/>
+    <sheet name="quality_of_surveillance" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -351,299 +353,1189 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ADMIN1 GEO_ID</t>
+          <t>Subnational level</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>GEO_ID</t>
+          <t>Municipality</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ADMIN1</t>
+          <t>Population immunity</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ADMIN2</t>
+          <t>Surveillance quality</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>INMUNIDAD_POB</t>
+          <t>Program delivery performance</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CALIDAD_VIG</t>
+          <t>Threat assessment</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>RENDIMIENTO_PROG</t>
+          <t>Rapid response</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>EVAL_AMENAZA</t>
+          <t>Risk points</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>RES_RAPIDA</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL_PR</t>
+          <t>Risk level</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BLZ.1_1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>12</v>
       </c>
       <c r="H2">
-        <v>9</v>
-      </c>
-      <c r="I2">
-        <v>12</v>
-      </c>
-      <c r="J2">
         <v>57</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BLZ.2_1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>CAYO</t>
         </is>
       </c>
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
       <c r="E3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
         <v>38</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BLZ.3_1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>COROZAL</t>
         </is>
       </c>
+      <c r="C4">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
       <c r="E4">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H4">
-        <v>7</v>
-      </c>
-      <c r="I4">
-        <v>12</v>
-      </c>
-      <c r="J4">
         <v>34</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BLZ.4_1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
           <t>ORANGE WALK</t>
         </is>
       </c>
+      <c r="C5">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
       <c r="E5">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H5">
-        <v>7</v>
-      </c>
-      <c r="I5">
-        <v>12</v>
-      </c>
-      <c r="J5">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BLZ.5_1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
           <t>STANN CREEK</t>
         </is>
       </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
       <c r="E6">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H6">
-        <v>7</v>
-      </c>
-      <c r="I6">
-        <v>6</v>
-      </c>
-      <c r="J6">
         <v>41</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BLZ</t>
+          <t>BELIZE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BLZ.6_1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>BELIZE</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
           <t>TOLEDO</t>
         </is>
       </c>
+      <c r="C7">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
       <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>30</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Subnational level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total risk points</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 coverage 2019 (%)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 coverage 2020 (%)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 coverage 2021 (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 coverage 2022 (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 coverage 2023 (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>MMR1 (Score)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MMR 2 coverage 2019 (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MMR 2 coverage 2020 (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>MMR 2 coverage 2021 (%)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>MMR 2 coverage 2022 (%)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>MMR 2 coverage 2023 (%)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>MMR2 (Score)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Campaign coverage (%)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>MR campaign (Score)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Unvaccinated suspected cases (%)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Unvaccinated suspected cases (Score)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Risk level</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <v>97</v>
+      </c>
+      <c r="E2">
+        <v>97</v>
+      </c>
+      <c r="F2">
+        <v>103</v>
+      </c>
+      <c r="G2">
+        <v>76</v>
+      </c>
+      <c r="H2">
+        <v>104</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>92</v>
+      </c>
+      <c r="K2">
+        <v>98</v>
+      </c>
+      <c r="L2">
+        <v>95</v>
+      </c>
+      <c r="M2">
+        <v>80</v>
+      </c>
+      <c r="N2">
+        <v>95</v>
+      </c>
+      <c r="O2">
+        <v>2</v>
+      </c>
+      <c r="P2">
+        <v>94</v>
+      </c>
+      <c r="Q2">
+        <v>2</v>
+      </c>
+      <c r="R2">
+        <v>37.5</v>
+      </c>
+      <c r="S2">
+        <v>10</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CAYO</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>94</v>
+      </c>
+      <c r="E3">
+        <v>92</v>
+      </c>
+      <c r="F3">
+        <v>88</v>
+      </c>
+      <c r="G3">
+        <v>89</v>
+      </c>
+      <c r="H3">
+        <v>92</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>86</v>
+      </c>
+      <c r="K3">
+        <v>90</v>
+      </c>
+      <c r="L3">
+        <v>96</v>
+      </c>
+      <c r="M3">
+        <v>89</v>
+      </c>
+      <c r="N3">
+        <v>84</v>
+      </c>
+      <c r="O3">
+        <v>3</v>
+      </c>
+      <c r="P3">
+        <v>93</v>
+      </c>
+      <c r="Q3">
+        <v>2</v>
+      </c>
+      <c r="R3">
+        <v>18.2</v>
+      </c>
+      <c r="S3">
+        <v>4</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COROZAL</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>95</v>
+      </c>
+      <c r="E4">
+        <v>99</v>
+      </c>
+      <c r="F4">
+        <v>102</v>
+      </c>
+      <c r="G4">
+        <v>122</v>
+      </c>
+      <c r="H4">
+        <v>94</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>94</v>
+      </c>
+      <c r="K4">
+        <v>94</v>
+      </c>
+      <c r="L4">
+        <v>100</v>
+      </c>
+      <c r="M4">
+        <v>108</v>
+      </c>
+      <c r="N4">
+        <v>93</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>97</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>33.3</v>
+      </c>
+      <c r="S4">
+        <v>10</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ORANGE WALK</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>96</v>
+      </c>
+      <c r="E5">
+        <v>98</v>
+      </c>
+      <c r="F5">
+        <v>110</v>
+      </c>
+      <c r="G5">
+        <v>100</v>
+      </c>
+      <c r="H5">
+        <v>98</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>96</v>
+      </c>
+      <c r="K5">
+        <v>98</v>
+      </c>
+      <c r="L5">
+        <v>97</v>
+      </c>
+      <c r="M5">
+        <v>96</v>
+      </c>
+      <c r="N5">
+        <v>97</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>88</v>
+      </c>
+      <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="R5">
+        <v>100</v>
+      </c>
+      <c r="S5">
+        <v>10</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>STANN CREEK</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>94</v>
+      </c>
+      <c r="E6">
+        <v>93</v>
+      </c>
+      <c r="F6">
+        <v>92</v>
+      </c>
+      <c r="G6">
+        <v>66</v>
+      </c>
+      <c r="H6">
+        <v>97</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>90</v>
+      </c>
+      <c r="K6">
+        <v>98</v>
+      </c>
+      <c r="L6">
+        <v>98</v>
+      </c>
+      <c r="M6">
+        <v>79</v>
+      </c>
+      <c r="N6">
+        <v>92</v>
+      </c>
+      <c r="O6">
+        <v>3</v>
+      </c>
+      <c r="P6">
+        <v>97</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>33.3</v>
+      </c>
+      <c r="S6">
+        <v>10</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TOLEDO</t>
+        </is>
+      </c>
+      <c r="C7">
         <v>13</v>
       </c>
+      <c r="D7">
+        <v>96</v>
+      </c>
+      <c r="E7">
+        <v>93</v>
+      </c>
       <c r="F7">
-        <v>4</v>
+        <v>82</v>
       </c>
       <c r="G7">
+        <v>117</v>
+      </c>
+      <c r="H7">
+        <v>94</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>92</v>
+      </c>
+      <c r="K7">
+        <v>97</v>
+      </c>
+      <c r="L7">
+        <v>90</v>
+      </c>
+      <c r="M7">
+        <v>84</v>
+      </c>
+      <c r="N7">
+        <v>82</v>
+      </c>
+      <c r="O7">
+        <v>3</v>
+      </c>
+      <c r="P7">
+        <v>88</v>
+      </c>
+      <c r="Q7">
+        <v>4</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>4</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Subnational level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Municipality</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total risk points</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Suspected cases</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Confirmed cases</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Annual rate of suspected cases (per 100,000 pop)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Annual rate of suspected cases (Score)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Cases with adequate investigation (%)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Cases with adequate investigation (Score)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Cases with adequate sample (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Cases with adequate sample (Score)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Samples received in laboratory in 5 days or less (%)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Samples received in laboratory in 5 days or less (Score)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Risk level</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>13</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>120600</v>
+      </c>
+      <c r="G2">
+        <v>10.8</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2">
+        <v>100</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>23.1</v>
+      </c>
+      <c r="N2">
+        <v>4</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CAYO</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>14</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>96197</v>
+      </c>
+      <c r="G3">
+        <v>14.6</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>100</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>100</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>21.4</v>
+      </c>
+      <c r="N3">
+        <v>4</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COROZAL</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
         <v>6</v>
       </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>48429</v>
+      </c>
+      <c r="G4">
+        <v>12.4</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>100</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>100</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>16.7</v>
+      </c>
+      <c r="N4">
+        <v>4</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ORANGE WALK</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>51749</v>
+      </c>
+      <c r="G5">
+        <v>1.9</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>100</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>100</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>4</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>STANN CREEK</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>43944</v>
+      </c>
+      <c r="G6">
+        <v>25</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>100</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>27.3</v>
+      </c>
+      <c r="N6">
+        <v>4</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BELIZE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TOLEDO</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <v>13</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>37614</v>
+      </c>
+      <c r="G7">
+        <v>34.6</v>
+      </c>
       <c r="H7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="J7">
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>100</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>30.8</v>
+      </c>
+      <c r="N7">
+        <v>4</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>